<commit_message>
Fix code reference in FRCoreMedicationProfile.fsh 8d9559f35171834289b92756246bbdea6a87551e
</commit_message>
<xml_diff>
--- a/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication.xlsx
+++ b/nr-doc-core-medication/ig/StructureDefinition-fr-core-medication.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2361" uniqueCount="379">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2216" uniqueCount="372">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-13T08:58:16+00:00</t>
+    <t>2026-08-13T09:15:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -767,10 +767,10 @@
     <t>Depending on the context of use, the code that was actually selected by the user (prescriber, dispenser, etc.) will have the coding.userSelected set to true.  As described in the coding datatype: "A coding may be marked as a "userSelected" if a user selected the particular coded value in a user interface (e.g. the user selects an item in a pick-list). If a user selected coding exists, it is the preferred choice for performing translations etc. Other codes can only be literal translations to alternative code systems, or codes at a lower level of granularity (e.g. a generic code for a vendor-specific primary one).</t>
   </si>
   <si>
-    <t>A coded concept that defines the type of a medication.</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/ValueSet/medication-codes|4.0.1</t>
+    <t>required</t>
+  </si>
+  <si>
+    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-medication-translation|2.2.0</t>
   </si>
   <si>
     <t>coding.code = //element(*,MedicationType)/DrugCoded/ProductCode@@ -789,76 +789,6 @@
     <t>RXO-1.1-Requested Give Code.code / RXE-2.1-Give Code.code / RXD-2.1-Dispense/Give Code.code / RXG-4.1-Give Code.code /RXA-5.1-Administered Code.code / RXC-2.1 Component Code</t>
   </si>
   <si>
-    <t>Medication.code.id</t>
-  </si>
-  <si>
-    <t>Medication.code.extension</t>
-  </si>
-  <si>
-    <t>Additional content defined by implementations</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>Medication.code.coding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coding
-</t>
-  </si>
-  <si>
-    <t>Code defined by a terminology system</t>
-  </si>
-  <si>
-    <t>A reference to a code defined by a terminology system.</t>
-  </si>
-  <si>
-    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
-  </si>
-  <si>
-    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
-  </si>
-  <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-medication-translation|2.2.0</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding</t>
-  </si>
-  <si>
-    <t>union(., ./translation)</t>
-  </si>
-  <si>
-    <t>C*E.1-8, C*E.10-22</t>
-  </si>
-  <si>
-    <t>Medication.code.text</t>
-  </si>
-  <si>
-    <t>Plain text representation of the concept</t>
-  </si>
-  <si>
-    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
-  </si>
-  <si>
-    <t>Very often the text is the same as a displayName of one of the codings.</t>
-  </si>
-  <si>
-    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>./originalText[mediaType/code="text/plain"]/data</t>
-  </si>
-  <si>
-    <t>C*E.9. But note many systems use C*E.2 for this</t>
-  </si>
-  <si>
     <t>Medication.status</t>
   </si>
   <si>
@@ -972,6 +902,12 @@
     <t>Medication.ingredient.extension</t>
   </si>
   <si>
+    <t>Additional content defined by implementations</t>
+  </si>
+  <si>
+    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
+  </si>
+  <si>
     <t>Medication.ingredient.modifierExtension</t>
   </si>
   <si>
@@ -1058,6 +994,31 @@
     <t>Medication.ingredient.item[x].coding</t>
   </si>
   <si>
+    <t xml:space="preserve">Coding
+</t>
+  </si>
+  <si>
+    <t>Code defined by a terminology system</t>
+  </si>
+  <si>
+    <t>A reference to a code defined by a terminology system.</t>
+  </si>
+  <si>
+    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
+  </si>
+  <si>
+    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>union(., ./translation)</t>
+  </si>
+  <si>
+    <t>C*E.1-8, C*E.10-22</t>
+  </si>
+  <si>
     <t>Medication.ingredient.item[x]:itemCodeableConcept.text</t>
   </si>
   <si>
@@ -1065,6 +1026,24 @@
   </si>
   <si>
     <t>Nom de la substance</t>
+  </si>
+  <si>
+    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
+  </si>
+  <si>
+    <t>Very often the text is the same as a displayName of one of the codings.</t>
+  </si>
+  <si>
+    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>./originalText[mediaType/code="text/plain"]/data</t>
+  </si>
+  <si>
+    <t>C*E.9. But note many systems use C*E.2 for this</t>
   </si>
   <si>
     <t>Medication.ingredient.isActive</t>
@@ -1513,7 +1492,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN65"/>
+  <dimension ref="A1:AN61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="54.796875" customWidth="true" bestFit="true"/>
@@ -5250,11 +5229,9 @@
         <v>78</v>
       </c>
       <c r="X33" t="s" s="2">
-        <v>204</v>
-      </c>
-      <c r="Y33" t="s" s="2">
         <v>239</v>
       </c>
+      <c r="Y33" s="2"/>
       <c r="Z33" t="s" s="2">
         <v>240</v>
       </c>
@@ -5323,21 +5300,23 @@
         <v>78</v>
       </c>
       <c r="I34" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>178</v>
+        <v>108</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>179</v>
+        <v>246</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>180</v>
-      </c>
-      <c r="N34" s="2"/>
+        <v>247</v>
+      </c>
+      <c r="N34" t="s" s="2">
+        <v>248</v>
+      </c>
       <c r="O34" s="2"/>
       <c r="P34" t="s" s="2">
         <v>78</v>
@@ -5362,13 +5341,13 @@
         <v>78</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>78</v>
+        <v>239</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>78</v>
+        <v>249</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>78</v>
+        <v>250</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>78</v>
@@ -5386,7 +5365,7 @@
         <v>78</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>181</v>
+        <v>245</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5398,13 +5377,13 @@
         <v>78</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="AK34" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>182</v>
+        <v>251</v>
       </c>
       <c r="AM34" t="s" s="2">
         <v>78</v>
@@ -5415,21 +5394,21 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>222</v>
+        <v>78</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>78</v>
@@ -5438,20 +5417,18 @@
         <v>78</v>
       </c>
       <c r="J35" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>133</v>
+        <v>253</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>225</v>
-      </c>
+        <v>255</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>78</v>
@@ -5488,51 +5465,51 @@
         <v>78</v>
       </c>
       <c r="AB35" t="s" s="2">
-        <v>136</v>
+        <v>78</v>
       </c>
       <c r="AC35" t="s" s="2">
-        <v>186</v>
+        <v>78</v>
       </c>
       <c r="AD35" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE35" t="s" s="2">
-        <v>137</v>
+        <v>78</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>187</v>
+        <v>252</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>78</v>
+        <v>256</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>182</v>
+        <v>257</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>78</v>
+        <v>258</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>78</v>
+        <v>259</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5543,7 +5520,7 @@
         <v>79</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>78</v>
@@ -5552,23 +5529,21 @@
         <v>78</v>
       </c>
       <c r="J36" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>250</v>
+        <v>201</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>253</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>254</v>
-      </c>
+        <v>263</v>
+      </c>
+      <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>78</v>
       </c>
@@ -5592,11 +5567,11 @@
         <v>78</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="Y36" s="2"/>
       <c r="Z36" t="s" s="2">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>78</v>
@@ -5614,13 +5589,13 @@
         <v>78</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>78</v>
@@ -5629,24 +5604,24 @@
         <v>100</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>78</v>
+        <v>265</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="AM36" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>259</v>
+        <v>267</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5669,20 +5644,16 @@
         <v>89</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>178</v>
+        <v>269</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="N37" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="O37" t="s" s="2">
-        <v>264</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>78</v>
       </c>
@@ -5730,7 +5701,7 @@
         <v>78</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
@@ -5748,21 +5719,21 @@
         <v>78</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>267</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5773,28 +5744,28 @@
         <v>79</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I38" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="J38" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>108</v>
+        <v>274</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -5820,37 +5791,37 @@
         <v>78</v>
       </c>
       <c r="X38" t="s" s="2">
-        <v>255</v>
+        <v>78</v>
       </c>
       <c r="Y38" t="s" s="2">
-        <v>272</v>
+        <v>78</v>
       </c>
       <c r="Z38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF38" t="s" s="2">
         <v>273</v>
       </c>
-      <c r="AA38" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB38" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC38" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD38" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE38" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF38" t="s" s="2">
-        <v>268</v>
-      </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>78</v>
@@ -5862,7 +5833,7 @@
         <v>78</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="AM38" t="s" s="2">
         <v>78</v>
@@ -5873,10 +5844,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5896,16 +5867,16 @@
         <v>78</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>276</v>
+        <v>178</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>277</v>
+        <v>179</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>278</v>
+        <v>180</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5956,7 +5927,7 @@
         <v>78</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>275</v>
+        <v>181</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>79</v>
@@ -5968,38 +5939,38 @@
         <v>78</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>279</v>
+        <v>78</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>280</v>
+        <v>182</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>281</v>
+        <v>78</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>282</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>78</v>
+        <v>222</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>78</v>
@@ -6011,16 +5982,16 @@
         <v>78</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>201</v>
+        <v>133</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>286</v>
+        <v>225</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
@@ -6046,11 +6017,13 @@
         <v>78</v>
       </c>
       <c r="X40" t="s" s="2">
-        <v>255</v>
-      </c>
-      <c r="Y40" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="Y40" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="Z40" t="s" s="2">
-        <v>287</v>
+        <v>78</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>78</v>
@@ -6068,71 +6041,75 @@
         <v>78</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>283</v>
+        <v>187</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>288</v>
+        <v>78</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>289</v>
+        <v>182</v>
       </c>
       <c r="AM40" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>290</v>
+        <v>78</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>78</v>
+        <v>284</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I41" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="J41" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>292</v>
+        <v>133</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>294</v>
-      </c>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
+        <v>286</v>
+      </c>
+      <c r="N41" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="O41" t="s" s="2">
+        <v>226</v>
+      </c>
       <c r="P41" t="s" s="2">
         <v>78</v>
       </c>
@@ -6180,25 +6157,25 @@
         <v>78</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>295</v>
+        <v>131</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>78</v>
@@ -6209,10 +6186,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6220,10 +6197,10 @@
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>78</v>
@@ -6235,18 +6212,18 @@
         <v>78</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>299</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>300</v>
-      </c>
-      <c r="O42" s="2"/>
+        <v>291</v>
+      </c>
+      <c r="N42" s="2"/>
+      <c r="O42" t="s" s="2">
+        <v>292</v>
+      </c>
       <c r="P42" t="s" s="2">
         <v>78</v>
       </c>
@@ -6282,25 +6259,23 @@
         <v>78</v>
       </c>
       <c r="AB42" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC42" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>293</v>
+      </c>
+      <c r="AC42" s="2"/>
       <c r="AD42" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE42" t="s" s="2">
-        <v>78</v>
+        <v>294</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>78</v>
@@ -6309,26 +6284,28 @@
         <v>100</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>78</v>
+        <v>241</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="AM42" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>78</v>
+        <v>296</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="C43" s="2"/>
+        <v>288</v>
+      </c>
+      <c r="C43" t="s" s="2">
+        <v>298</v>
+      </c>
       <c r="D43" t="s" s="2">
         <v>78</v>
       </c>
@@ -6349,16 +6326,18 @@
         <v>78</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>178</v>
+        <v>299</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>179</v>
+        <v>290</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>180</v>
+        <v>291</v>
       </c>
       <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
+      <c r="O43" t="s" s="2">
+        <v>292</v>
+      </c>
       <c r="P43" t="s" s="2">
         <v>78</v>
       </c>
@@ -6406,10 +6385,10 @@
         <v>78</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>181</v>
+        <v>288</v>
       </c>
       <c r="AG43" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AH43" t="s" s="2">
         <v>88</v>
@@ -6418,38 +6397,40 @@
         <v>78</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>78</v>
+        <v>241</v>
       </c>
       <c r="AL43" t="s" s="2">
-        <v>182</v>
+        <v>295</v>
       </c>
       <c r="AM43" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>78</v>
+        <v>296</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="C44" s="2"/>
+        <v>288</v>
+      </c>
+      <c r="C44" t="s" s="2">
+        <v>301</v>
+      </c>
       <c r="D44" t="s" s="2">
-        <v>222</v>
+        <v>78</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G44" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H44" t="s" s="2">
         <v>78</v>
@@ -6461,18 +6442,18 @@
         <v>78</v>
       </c>
       <c r="K44" t="s" s="2">
-        <v>133</v>
+        <v>201</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>247</v>
+        <v>302</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="O44" s="2"/>
+        <v>291</v>
+      </c>
+      <c r="N44" s="2"/>
+      <c r="O44" t="s" s="2">
+        <v>292</v>
+      </c>
       <c r="P44" t="s" s="2">
         <v>78</v>
       </c>
@@ -6496,13 +6477,11 @@
         <v>78</v>
       </c>
       <c r="X44" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y44" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>239</v>
+      </c>
+      <c r="Y44" s="2"/>
       <c r="Z44" t="s" s="2">
-        <v>78</v>
+        <v>303</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>78</v>
@@ -6520,31 +6499,31 @@
         <v>78</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>187</v>
+        <v>288</v>
       </c>
       <c r="AG44" t="s" s="2">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="AH44" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI44" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>78</v>
+        <v>241</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>182</v>
+        <v>295</v>
       </c>
       <c r="AM44" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN44" t="s" s="2">
-        <v>78</v>
+        <v>296</v>
       </c>
     </row>
     <row r="45">
@@ -6552,43 +6531,39 @@
         <v>304</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>305</v>
+        <v>78</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I45" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>133</v>
+        <v>178</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>306</v>
+        <v>179</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="N45" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="O45" t="s" s="2">
-        <v>226</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>78</v>
       </c>
@@ -6636,25 +6611,25 @@
         <v>78</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>308</v>
+        <v>181</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI45" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>139</v>
+        <v>78</v>
       </c>
       <c r="AK45" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>131</v>
+        <v>182</v>
       </c>
       <c r="AM45" t="s" s="2">
         <v>78</v>
@@ -6665,21 +6640,21 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>78</v>
+        <v>222</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G46" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H46" t="s" s="2">
         <v>78</v>
@@ -6691,18 +6666,18 @@
         <v>78</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>310</v>
+        <v>133</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>311</v>
+        <v>281</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="N46" s="2"/>
-      <c r="O46" t="s" s="2">
-        <v>313</v>
-      </c>
+        <v>282</v>
+      </c>
+      <c r="N46" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>78</v>
       </c>
@@ -6738,53 +6713,53 @@
         <v>78</v>
       </c>
       <c r="AB46" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="AC46" s="2"/>
+        <v>136</v>
+      </c>
+      <c r="AC46" t="s" s="2">
+        <v>186</v>
+      </c>
       <c r="AD46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE46" t="s" s="2">
-        <v>315</v>
+        <v>137</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>309</v>
+        <v>187</v>
       </c>
       <c r="AG46" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AH46" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>241</v>
+        <v>78</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>316</v>
+        <v>182</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>317</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="B47" t="s" s="2">
         <v>309</v>
       </c>
-      <c r="C47" t="s" s="2">
-        <v>319</v>
-      </c>
+      <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
         <v>78</v>
       </c>
@@ -6793,7 +6768,7 @@
         <v>79</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>78</v>
@@ -6802,10 +6777,10 @@
         <v>78</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="L47" t="s" s="2">
         <v>311</v>
@@ -6813,9 +6788,11 @@
       <c r="M47" t="s" s="2">
         <v>312</v>
       </c>
-      <c r="N47" s="2"/>
+      <c r="N47" t="s" s="2">
+        <v>313</v>
+      </c>
       <c r="O47" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="P47" t="s" s="2">
         <v>78</v>
@@ -6864,13 +6841,13 @@
         <v>78</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="AG47" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI47" t="s" s="2">
         <v>78</v>
@@ -6879,7 +6856,7 @@
         <v>100</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>241</v>
+        <v>78</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>316</v>
@@ -6893,14 +6870,12 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="C48" t="s" s="2">
-        <v>322</v>
-      </c>
+        <v>319</v>
+      </c>
+      <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
         <v>78</v>
       </c>
@@ -6918,20 +6893,22 @@
         <v>78</v>
       </c>
       <c r="J48" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>201</v>
+        <v>178</v>
       </c>
       <c r="L48" t="s" s="2">
+        <v>320</v>
+      </c>
+      <c r="M48" t="s" s="2">
+        <v>321</v>
+      </c>
+      <c r="N48" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="O48" t="s" s="2">
         <v>323</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="N48" s="2"/>
-      <c r="O48" t="s" s="2">
-        <v>313</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>78</v>
@@ -6956,32 +6933,34 @@
         <v>78</v>
       </c>
       <c r="X48" t="s" s="2">
-        <v>255</v>
-      </c>
-      <c r="Y48" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="Y48" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="Z48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE48" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF48" t="s" s="2">
         <v>324</v>
       </c>
-      <c r="AA48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF48" t="s" s="2">
-        <v>309</v>
-      </c>
       <c r="AG48" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="AH48" t="s" s="2">
         <v>88</v>
@@ -6993,24 +6972,24 @@
         <v>100</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>241</v>
+        <v>78</v>
       </c>
       <c r="AL48" t="s" s="2">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="AM48" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>317</v>
+        <v>326</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7033,16 +7012,18 @@
         <v>78</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>178</v>
+        <v>328</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>179</v>
+        <v>329</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>180</v>
+        <v>330</v>
       </c>
       <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
+      <c r="O49" t="s" s="2">
+        <v>331</v>
+      </c>
       <c r="P49" t="s" s="2">
         <v>78</v>
       </c>
@@ -7090,7 +7071,7 @@
         <v>78</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>181</v>
+        <v>327</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>79</v>
@@ -7102,13 +7083,13 @@
         <v>78</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="AK49" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL49" t="s" s="2">
-        <v>182</v>
+        <v>332</v>
       </c>
       <c r="AM49" t="s" s="2">
         <v>78</v>
@@ -7119,21 +7100,21 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
-        <v>222</v>
+        <v>78</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G50" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H50" t="s" s="2">
         <v>78</v>
@@ -7145,17 +7126,15 @@
         <v>78</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>133</v>
+        <v>269</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>247</v>
+        <v>334</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N50" t="s" s="2">
-        <v>225</v>
-      </c>
+        <v>335</v>
+      </c>
+      <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
         <v>78</v>
@@ -7192,51 +7171,51 @@
         <v>78</v>
       </c>
       <c r="AB50" t="s" s="2">
-        <v>136</v>
+        <v>78</v>
       </c>
       <c r="AC50" t="s" s="2">
-        <v>186</v>
+        <v>78</v>
       </c>
       <c r="AD50" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE50" t="s" s="2">
-        <v>137</v>
+        <v>78</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>187</v>
+        <v>333</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH50" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI50" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ50" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>78</v>
+        <v>336</v>
       </c>
       <c r="AL50" t="s" s="2">
-        <v>182</v>
+        <v>272</v>
       </c>
       <c r="AM50" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN50" t="s" s="2">
-        <v>78</v>
+        <v>337</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7247,7 +7226,7 @@
         <v>79</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>78</v>
@@ -7256,23 +7235,19 @@
         <v>78</v>
       </c>
       <c r="J51" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>250</v>
+        <v>178</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>251</v>
+        <v>179</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>252</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>253</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>254</v>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="N51" s="2"/>
+      <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
         <v>78</v>
       </c>
@@ -7320,50 +7295,50 @@
         <v>78</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>257</v>
+        <v>181</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI51" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>100</v>
+        <v>78</v>
       </c>
       <c r="AK51" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL51" t="s" s="2">
-        <v>258</v>
+        <v>182</v>
       </c>
       <c r="AM51" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN51" t="s" s="2">
-        <v>259</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>78</v>
+        <v>222</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G52" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H52" t="s" s="2">
         <v>78</v>
@@ -7372,23 +7347,21 @@
         <v>78</v>
       </c>
       <c r="J52" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>178</v>
+        <v>133</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>333</v>
+        <v>281</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>262</v>
+        <v>282</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="O52" t="s" s="2">
-        <v>264</v>
-      </c>
+        <v>225</v>
+      </c>
+      <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
         <v>78</v>
       </c>
@@ -7424,53 +7397,55 @@
         <v>78</v>
       </c>
       <c r="AB52" t="s" s="2">
-        <v>78</v>
+        <v>136</v>
       </c>
       <c r="AC52" t="s" s="2">
-        <v>78</v>
+        <v>186</v>
       </c>
       <c r="AD52" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE52" t="s" s="2">
-        <v>78</v>
+        <v>137</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>265</v>
+        <v>187</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH52" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI52" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ52" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK52" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL52" t="s" s="2">
-        <v>266</v>
+        <v>182</v>
       </c>
       <c r="AM52" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN52" t="s" s="2">
-        <v>267</v>
+        <v>78</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="C53" s="2"/>
+        <v>339</v>
+      </c>
+      <c r="C53" t="s" s="2">
+        <v>341</v>
+      </c>
       <c r="D53" t="s" s="2">
         <v>78</v>
       </c>
@@ -7491,18 +7466,16 @@
         <v>78</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="N53" s="2"/>
-      <c r="O53" t="s" s="2">
-        <v>338</v>
-      </c>
+      <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
         <v>78</v>
       </c>
@@ -7550,25 +7523,25 @@
         <v>78</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>334</v>
+        <v>187</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH53" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI53" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ53" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK53" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL53" t="s" s="2">
-        <v>339</v>
+        <v>78</v>
       </c>
       <c r="AM53" t="s" s="2">
         <v>78</v>
@@ -7579,10 +7552,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7602,16 +7575,16 @@
         <v>78</v>
       </c>
       <c r="J54" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>292</v>
+        <v>214</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -7662,7 +7635,7 @@
         <v>78</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>79</v>
@@ -7677,24 +7650,24 @@
         <v>100</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>343</v>
+        <v>78</v>
       </c>
       <c r="AL54" t="s" s="2">
-        <v>295</v>
+        <v>349</v>
       </c>
       <c r="AM54" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>344</v>
+        <v>78</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -7714,16 +7687,16 @@
         <v>78</v>
       </c>
       <c r="J55" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>178</v>
+        <v>214</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>179</v>
+        <v>351</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>180</v>
+        <v>352</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -7774,7 +7747,7 @@
         <v>78</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>181</v>
+        <v>353</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>79</v>
@@ -7786,13 +7759,13 @@
         <v>78</v>
       </c>
       <c r="AJ55" t="s" s="2">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="AK55" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL55" t="s" s="2">
-        <v>182</v>
+        <v>354</v>
       </c>
       <c r="AM55" t="s" s="2">
         <v>78</v>
@@ -7803,21 +7776,21 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
-        <v>222</v>
+        <v>78</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" t="s" s="2">
         <v>79</v>
       </c>
       <c r="G56" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="H56" t="s" s="2">
         <v>78</v>
@@ -7829,17 +7802,15 @@
         <v>78</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>133</v>
+        <v>274</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>247</v>
+        <v>356</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N56" t="s" s="2">
-        <v>225</v>
-      </c>
+        <v>357</v>
+      </c>
+      <c r="N56" s="2"/>
       <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
         <v>78</v>
@@ -7876,37 +7847,37 @@
         <v>78</v>
       </c>
       <c r="AB56" t="s" s="2">
-        <v>136</v>
+        <v>78</v>
       </c>
       <c r="AC56" t="s" s="2">
-        <v>186</v>
+        <v>78</v>
       </c>
       <c r="AD56" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AE56" t="s" s="2">
-        <v>137</v>
+        <v>78</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>187</v>
+        <v>355</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH56" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI56" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ56" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>78</v>
+        <v>256</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>182</v>
+        <v>358</v>
       </c>
       <c r="AM56" t="s" s="2">
         <v>78</v>
@@ -7917,14 +7888,12 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>346</v>
-      </c>
-      <c r="C57" t="s" s="2">
-        <v>348</v>
-      </c>
+        <v>359</v>
+      </c>
+      <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
         <v>78</v>
       </c>
@@ -7945,13 +7914,13 @@
         <v>78</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>349</v>
+        <v>178</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>350</v>
+        <v>179</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>351</v>
+        <v>180</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -8002,25 +7971,25 @@
         <v>78</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH57" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="AI57" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>139</v>
+        <v>78</v>
       </c>
       <c r="AK57" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL57" t="s" s="2">
-        <v>78</v>
+        <v>182</v>
       </c>
       <c r="AM57" t="s" s="2">
         <v>78</v>
@@ -8031,21 +8000,21 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
-        <v>78</v>
+        <v>222</v>
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G58" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H58" t="s" s="2">
         <v>78</v>
@@ -8054,18 +8023,20 @@
         <v>78</v>
       </c>
       <c r="J58" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>214</v>
+        <v>133</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>353</v>
+        <v>281</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>354</v>
-      </c>
-      <c r="N58" s="2"/>
+        <v>282</v>
+      </c>
+      <c r="N58" t="s" s="2">
+        <v>225</v>
+      </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
         <v>78</v>
@@ -8114,25 +8085,25 @@
         <v>78</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>355</v>
+        <v>187</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH58" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI58" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK58" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL58" t="s" s="2">
-        <v>356</v>
+        <v>182</v>
       </c>
       <c r="AM58" t="s" s="2">
         <v>78</v>
@@ -8143,42 +8114,46 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
-        <v>78</v>
+        <v>284</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s" s="2">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="G59" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="H59" t="s" s="2">
         <v>78</v>
       </c>
       <c r="I59" t="s" s="2">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="J59" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>214</v>
+        <v>133</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>358</v>
+        <v>285</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>359</v>
-      </c>
-      <c r="N59" s="2"/>
-      <c r="O59" s="2"/>
+        <v>286</v>
+      </c>
+      <c r="N59" t="s" s="2">
+        <v>225</v>
+      </c>
+      <c r="O59" t="s" s="2">
+        <v>226</v>
+      </c>
       <c r="P59" t="s" s="2">
         <v>78</v>
       </c>
@@ -8226,25 +8201,25 @@
         <v>78</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>360</v>
+        <v>287</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AH59" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AI59" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK59" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AL59" t="s" s="2">
-        <v>361</v>
+        <v>131</v>
       </c>
       <c r="AM59" t="s" s="2">
         <v>78</v>
@@ -8281,7 +8256,7 @@
         <v>78</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>297</v>
+        <v>178</v>
       </c>
       <c r="L60" t="s" s="2">
         <v>363</v>
@@ -8353,16 +8328,16 @@
         <v>100</v>
       </c>
       <c r="AK60" t="s" s="2">
-        <v>279</v>
+        <v>256</v>
       </c>
       <c r="AL60" t="s" s="2">
+        <v>233</v>
+      </c>
+      <c r="AM60" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AN60" t="s" s="2">
         <v>365</v>
-      </c>
-      <c r="AM60" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN60" t="s" s="2">
-        <v>78</v>
       </c>
     </row>
     <row r="61">
@@ -8393,13 +8368,13 @@
         <v>78</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>178</v>
+        <v>367</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>179</v>
+        <v>368</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>180</v>
+        <v>369</v>
       </c>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
@@ -8450,7 +8425,7 @@
         <v>78</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>181</v>
+        <v>366</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>79</v>
@@ -8462,473 +8437,19 @@
         <v>78</v>
       </c>
       <c r="AJ61" t="s" s="2">
-        <v>78</v>
+        <v>100</v>
       </c>
       <c r="AK61" t="s" s="2">
-        <v>78</v>
+        <v>256</v>
       </c>
       <c r="AL61" t="s" s="2">
-        <v>182</v>
+        <v>370</v>
       </c>
       <c r="AM61" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="s" s="2">
-        <v>367</v>
-      </c>
-      <c r="B62" t="s" s="2">
-        <v>367</v>
-      </c>
-      <c r="C62" s="2"/>
-      <c r="D62" t="s" s="2">
-        <v>222</v>
-      </c>
-      <c r="E62" s="2"/>
-      <c r="F62" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K62" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="L62" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="N62" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="O62" s="2"/>
-      <c r="P62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q62" s="2"/>
-      <c r="R62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF62" t="s" s="2">
-        <v>187</v>
-      </c>
-      <c r="AG62" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH62" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AI62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ62" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AK62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL62" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="AM62" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN62" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="s" s="2">
-        <v>368</v>
-      </c>
-      <c r="B63" t="s" s="2">
-        <v>368</v>
-      </c>
-      <c r="C63" s="2"/>
-      <c r="D63" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="E63" s="2"/>
-      <c r="F63" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G63" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I63" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="J63" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="K63" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="L63" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="M63" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="N63" t="s" s="2">
-        <v>225</v>
-      </c>
-      <c r="O63" t="s" s="2">
-        <v>226</v>
-      </c>
-      <c r="P63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q63" s="2"/>
-      <c r="R63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF63" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="AG63" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH63" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AI63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ63" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="AK63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AL63" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="AM63" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN63" t="s" s="2">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="s" s="2">
-        <v>369</v>
-      </c>
-      <c r="B64" t="s" s="2">
-        <v>369</v>
-      </c>
-      <c r="C64" s="2"/>
-      <c r="D64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E64" s="2"/>
-      <c r="F64" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G64" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K64" t="s" s="2">
-        <v>178</v>
-      </c>
-      <c r="L64" t="s" s="2">
-        <v>370</v>
-      </c>
-      <c r="M64" t="s" s="2">
         <v>371</v>
-      </c>
-      <c r="N64" s="2"/>
-      <c r="O64" s="2"/>
-      <c r="P64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q64" s="2"/>
-      <c r="R64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF64" t="s" s="2">
-        <v>369</v>
-      </c>
-      <c r="AG64" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH64" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ64" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK64" t="s" s="2">
-        <v>279</v>
-      </c>
-      <c r="AL64" t="s" s="2">
-        <v>233</v>
-      </c>
-      <c r="AM64" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN64" t="s" s="2">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="s" s="2">
-        <v>373</v>
-      </c>
-      <c r="B65" t="s" s="2">
-        <v>373</v>
-      </c>
-      <c r="C65" s="2"/>
-      <c r="D65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="E65" s="2"/>
-      <c r="F65" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="G65" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="I65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="J65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="K65" t="s" s="2">
-        <v>374</v>
-      </c>
-      <c r="L65" t="s" s="2">
-        <v>375</v>
-      </c>
-      <c r="M65" t="s" s="2">
-        <v>376</v>
-      </c>
-      <c r="N65" s="2"/>
-      <c r="O65" s="2"/>
-      <c r="P65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Q65" s="2"/>
-      <c r="R65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="S65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="T65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="U65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="V65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="W65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="X65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Z65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AA65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AB65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AC65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AD65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AF65" t="s" s="2">
-        <v>373</v>
-      </c>
-      <c r="AG65" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AH65" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AJ65" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK65" t="s" s="2">
-        <v>279</v>
-      </c>
-      <c r="AL65" t="s" s="2">
-        <v>377</v>
-      </c>
-      <c r="AM65" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AN65" t="s" s="2">
-        <v>378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>